<commit_message>
Updates names in schedule
</commit_message>
<xml_diff>
--- a/docs/schedule.xlsx
+++ b/docs/schedule.xlsx
@@ -1,25 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jenfra/NBISCourses/scRNAseq/workshop-scRNAseq/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jenfra/NBISCourses/scRNAseq/workshop-scRNAseq/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A131CE26-ACD8-8E47-BA54-BDA7C998D97B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD10540-D4BE-BB4B-8F50-A093DDAA5C32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1420" yWindow="1440" windowWidth="35000" windowHeight="21100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15420" yWindow="5620" windowWidth="35000" windowHeight="21100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="schedule" localSheetId="0">Sheet1!$A$1:$L$42</definedName>
+    <definedName name="schedule" localSheetId="0">Sheet1!$A$1:$L$41</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -28,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="82">
   <si>
     <t>date</t>
   </si>
@@ -117,9 +128,6 @@
     <t>Lecture: Dimensionality reduction</t>
   </si>
   <si>
-    <t>Nikolay Oskolkov</t>
-  </si>
-  <si>
     <t>lectures/dimred.pdf</t>
   </si>
   <si>
@@ -144,15 +152,6 @@
     <t>Lab: Clustering</t>
   </si>
   <si>
-    <t>Lecture: Single Cell Epigenetics</t>
-  </si>
-  <si>
-    <t>Jakub Westholm</t>
-  </si>
-  <si>
-    <t>lectures/atacseq.pdf</t>
-  </si>
-  <si>
     <t>Lecture: Differential Gene Expression</t>
   </si>
   <si>
@@ -177,9 +176,6 @@
     <t>Lecture: Trajectory inference</t>
   </si>
   <si>
-    <t>Paulo Czarnewski</t>
-  </si>
-  <si>
     <t>lectures/trajectory.pdf</t>
   </si>
   <si>
@@ -204,24 +200,6 @@
     <t>zoom</t>
   </si>
   <si>
-    <t>10/04/2025</t>
-  </si>
-  <si>
-    <t>03/04/2025</t>
-  </si>
-  <si>
-    <t>02/04/2025</t>
-  </si>
-  <si>
-    <t>01/04/2025</t>
-  </si>
-  <si>
-    <t>31/03/2025</t>
-  </si>
-  <si>
-    <t>ÅB, SR, JF</t>
-  </si>
-  <si>
     <t>Presentation of projects</t>
   </si>
   <si>
@@ -270,44 +248,50 @@
     <t>lectures/BYOD_intro.pdf</t>
   </si>
   <si>
-    <t>https://youtu.be/OccS8ZFN0E4</t>
-  </si>
-  <si>
-    <t>https://youtu.be/gAAs4BWfAtM</t>
-  </si>
-  <si>
-    <t>https://youtu.be/23C5LFXZZ2U</t>
-  </si>
-  <si>
-    <t>https://youtu.be/X6zQ0a0da8I</t>
-  </si>
-  <si>
-    <t>https://youtu.be/a-vzYSYA9mg</t>
-  </si>
-  <si>
-    <t>https://youtu.be/7D6iMgvPFZk</t>
-  </si>
-  <si>
-    <t>https://youtu.be/FvIsISt8Auw</t>
-  </si>
-  <si>
-    <t>https://youtu.be/-DnF0uD3euo</t>
-  </si>
-  <si>
-    <t>https://youtu.be/lGAcQqeEOzA</t>
-  </si>
-  <si>
-    <t>https://youtu.be/h8XZzdBMokc</t>
-  </si>
-  <si>
-    <t>https://youtu.be/epN5KSt6qZg</t>
+    <t>SR, JF</t>
+  </si>
+  <si>
+    <t>Yuan Li</t>
+  </si>
+  <si>
+    <t>Stefan Ebmeyer</t>
+  </si>
+  <si>
+    <t>Lecture: Cell-Cell Communication</t>
+  </si>
+  <si>
+    <t>lectures/ccc.pdf</t>
+  </si>
+  <si>
+    <t>Jose Liñares-Blanco</t>
+  </si>
+  <si>
+    <t>27/04/2026</t>
+  </si>
+  <si>
+    <t>13/04/2025</t>
+  </si>
+  <si>
+    <t>14/04/2025</t>
+  </si>
+  <si>
+    <t>15/04/2025</t>
+  </si>
+  <si>
+    <t>16/04/2025</t>
+  </si>
+  <si>
+    <t>Susanne Reinsbach</t>
+  </si>
+  <si>
+    <t>Aditya Singh</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -319,6 +303,12 @@
       <u/>
       <sz val="12"/>
       <color rgb="FF0563C1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -738,7 +728,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="9.6640625" customWidth="1"/>
@@ -794,10 +784,10 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C2" s="2">
         <v>0.375</v>
@@ -809,7 +799,7 @@
         <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>14</v>
@@ -824,7 +814,7 @@
         <v>0.4375</v>
       </c>
       <c r="E3" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="F3" t="s">
         <v>18</v>
@@ -832,9 +822,7 @@
       <c r="H3" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>80</v>
-      </c>
+      <c r="K3" s="3"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="C4" s="2">
@@ -863,9 +851,7 @@
       <c r="H5" t="s">
         <v>16</v>
       </c>
-      <c r="K5" s="4" t="s">
-        <v>81</v>
-      </c>
+      <c r="K5" s="4"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="C6" s="2">
@@ -889,7 +875,7 @@
         <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>13</v>
+        <v>69</v>
       </c>
       <c r="H7" t="s">
         <v>22</v>
@@ -907,7 +893,7 @@
         <v>23</v>
       </c>
       <c r="F8" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="I8" t="s">
         <v>24</v>
@@ -935,13 +921,10 @@
         <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="H10" t="s">
         <v>26</v>
-      </c>
-      <c r="K10" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
@@ -955,15 +938,15 @@
         <v>27</v>
       </c>
       <c r="F11" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="C12" s="2">
         <v>0.375</v>
@@ -975,14 +958,12 @@
         <v>28</v>
       </c>
       <c r="F12" t="s">
+        <v>80</v>
+      </c>
+      <c r="H12" t="s">
         <v>29</v>
       </c>
-      <c r="H12" t="s">
-        <v>30</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>83</v>
-      </c>
+      <c r="K12" s="3"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="C13" s="2">
@@ -1003,10 +984,10 @@
         <v>0.5</v>
       </c>
       <c r="E14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F14" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="I14" t="s">
         <v>24</v>
@@ -1032,17 +1013,15 @@
         <v>0.58333333333333304</v>
       </c>
       <c r="E16" t="s">
+        <v>31</v>
+      </c>
+      <c r="F16" t="s">
+        <v>81</v>
+      </c>
+      <c r="H16" t="s">
         <v>32</v>
       </c>
-      <c r="F16" t="s">
-        <v>29</v>
-      </c>
-      <c r="H16" t="s">
-        <v>33</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>84</v>
-      </c>
+      <c r="K16" s="3"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C17" s="2">
@@ -1052,10 +1031,10 @@
         <v>0.625</v>
       </c>
       <c r="E17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F17" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
       <c r="I17" t="s">
         <v>24</v>
@@ -1081,16 +1060,13 @@
         <v>0.6875</v>
       </c>
       <c r="E19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F19" t="s">
         <v>13</v>
       </c>
       <c r="H19" t="s">
-        <v>36</v>
-      </c>
-      <c r="K19" t="s">
-        <v>85</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
@@ -1104,445 +1080,429 @@
         <v>27</v>
       </c>
       <c r="F20" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
+      <c r="A21" t="s">
+        <v>78</v>
+      </c>
+      <c r="C21" s="2">
+        <v>0.375</v>
+      </c>
+      <c r="D21" s="2">
+        <v>0.41666666666666702</v>
+      </c>
+      <c r="E21" t="s">
+        <v>36</v>
+      </c>
+      <c r="F21" t="s">
+        <v>80</v>
+      </c>
+      <c r="I21" t="s">
+        <v>24</v>
+      </c>
+      <c r="K21" s="3"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>60</v>
-      </c>
       <c r="C22" s="2">
-        <v>0.375</v>
+        <v>0.41666666666666702</v>
       </c>
       <c r="D22" s="2">
-        <v>0.41666666666666702</v>
+        <v>0.4375</v>
       </c>
       <c r="E22" t="s">
-        <v>37</v>
-      </c>
-      <c r="F22" t="s">
-        <v>13</v>
-      </c>
-      <c r="I22" t="s">
-        <v>24</v>
-      </c>
-      <c r="K22" s="3"/>
+        <v>17</v>
+      </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C23" s="2">
-        <v>0.41666666666666702</v>
+        <v>0.4375</v>
       </c>
       <c r="D23" s="2">
-        <v>0.4375</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="E23" t="s">
-        <v>17</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="F23" t="s">
+        <v>55</v>
+      </c>
+      <c r="H23" t="s">
+        <v>38</v>
+      </c>
+      <c r="I23" t="s">
+        <v>64</v>
+      </c>
+      <c r="K23" s="3"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C24" s="2">
-        <v>0.4375</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D24" s="2">
-        <v>0.47916666666666669</v>
+        <v>0.5</v>
       </c>
       <c r="E24" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F24" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="H24" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="I24" t="s">
-        <v>75</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>86</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="K24" s="3"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C25" s="2">
-        <v>0.47916666666666669</v>
+        <v>0.5</v>
       </c>
       <c r="D25" s="2">
-        <v>0.5</v>
+        <v>0.54166666666666696</v>
       </c>
       <c r="E25" t="s">
-        <v>43</v>
-      </c>
-      <c r="F25" t="s">
-        <v>66</v>
-      </c>
-      <c r="H25" t="s">
-        <v>56</v>
-      </c>
-      <c r="I25" t="s">
-        <v>76</v>
-      </c>
-      <c r="K25" s="3" t="s">
-        <v>87</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="K25" s="3"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C26" s="2">
-        <v>0.5</v>
+        <v>0.54166666666666696</v>
       </c>
       <c r="D26" s="2">
-        <v>0.54166666666666696</v>
+        <v>0.58333333333333304</v>
       </c>
       <c r="E26" t="s">
-        <v>20</v>
-      </c>
-      <c r="K26" s="3"/>
+        <v>72</v>
+      </c>
+      <c r="F26" t="s">
+        <v>74</v>
+      </c>
+      <c r="H26" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C27" s="2">
-        <v>0.54166666666666696</v>
+        <v>0.58333333333333304</v>
       </c>
       <c r="D27" s="2">
-        <v>0.58333333333333304</v>
+        <v>0.60416666666666696</v>
       </c>
       <c r="E27" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F27" t="s">
-        <v>39</v>
-      </c>
-      <c r="H27" t="s">
-        <v>40</v>
-      </c>
-      <c r="K27" t="s">
-        <v>88</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="I27" t="s">
+        <v>24</v>
+      </c>
+      <c r="K27" s="3"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C28" s="2">
-        <v>0.58333333333333304</v>
+        <v>0.60416666666666696</v>
       </c>
       <c r="D28" s="2">
-        <v>0.60416666666666696</v>
+        <v>0.625</v>
       </c>
       <c r="E28" t="s">
-        <v>44</v>
-      </c>
-      <c r="F28" t="s">
-        <v>66</v>
-      </c>
-      <c r="I28" t="s">
-        <v>24</v>
-      </c>
-      <c r="K28" s="3"/>
+        <v>17</v>
+      </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C29" s="2">
-        <v>0.60416666666666696</v>
+        <v>0.625</v>
       </c>
       <c r="D29" s="2">
-        <v>0.625</v>
+        <v>0.6875</v>
       </c>
       <c r="E29" t="s">
-        <v>17</v>
+        <v>40</v>
+      </c>
+      <c r="F29" t="s">
+        <v>55</v>
+      </c>
+      <c r="I29" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C30" s="2">
-        <v>0.625</v>
+        <v>0.6875</v>
       </c>
       <c r="D30" s="2">
-        <v>0.6875</v>
+        <v>0.70833333333333304</v>
       </c>
       <c r="E30" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="F30" t="s">
-        <v>66</v>
-      </c>
-      <c r="I30" t="s">
-        <v>24</v>
+        <v>69</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>79</v>
+      </c>
       <c r="C31" s="2">
-        <v>0.6875</v>
+        <v>0.375</v>
       </c>
       <c r="D31" s="2">
-        <v>0.70833333333333304</v>
+        <v>0.41666666666666702</v>
       </c>
       <c r="E31" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="F31" t="s">
-        <v>63</v>
-      </c>
-      <c r="J31" s="3" t="s">
-        <v>72</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="H31" t="s">
+        <v>42</v>
+      </c>
+      <c r="K31" s="3"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>59</v>
-      </c>
       <c r="C32" s="2">
-        <v>0.375</v>
+        <v>0.41666666666666702</v>
       </c>
       <c r="D32" s="2">
-        <v>0.41666666666666702</v>
+        <v>0.4375</v>
       </c>
       <c r="E32" t="s">
-        <v>45</v>
-      </c>
-      <c r="F32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H32" t="s">
-        <v>46</v>
-      </c>
-      <c r="K32" s="3" t="s">
-        <v>89</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C33" s="2">
-        <v>0.41666666666666702</v>
+        <v>0.4375</v>
       </c>
       <c r="D33" s="2">
-        <v>0.4375</v>
+        <v>0.5</v>
       </c>
       <c r="E33" t="s">
-        <v>17</v>
+        <v>43</v>
+      </c>
+      <c r="F33" t="s">
+        <v>56</v>
+      </c>
+      <c r="I33" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C34" s="2">
-        <v>0.4375</v>
+        <v>0.5</v>
       </c>
       <c r="D34" s="2">
-        <v>0.5</v>
+        <v>0.54166666666666696</v>
       </c>
       <c r="E34" t="s">
-        <v>47</v>
-      </c>
-      <c r="F34" t="s">
-        <v>67</v>
-      </c>
-      <c r="I34" t="s">
-        <v>24</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="K34" s="3"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C35" s="2">
-        <v>0.5</v>
+        <v>0.54166666666666696</v>
       </c>
       <c r="D35" s="2">
-        <v>0.54166666666666696</v>
+        <v>0.58333333333333304</v>
       </c>
       <c r="E35" t="s">
-        <v>20</v>
-      </c>
-      <c r="K35" s="3"/>
+        <v>44</v>
+      </c>
+      <c r="F35" t="s">
+        <v>71</v>
+      </c>
+      <c r="H35" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C36" s="2">
-        <v>0.54166666666666696</v>
+        <v>0.58333333333333304</v>
       </c>
       <c r="D36" s="2">
-        <v>0.58333333333333304</v>
+        <v>0.64583333333333337</v>
       </c>
       <c r="E36" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F36" t="s">
-        <v>49</v>
-      </c>
-      <c r="H36" t="s">
-        <v>50</v>
-      </c>
-      <c r="K36" t="s">
-        <v>90</v>
+        <v>71</v>
+      </c>
+      <c r="I36" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C37" s="2">
-        <v>0.58333333333333304</v>
+        <v>0.64583333333333337</v>
       </c>
       <c r="D37" s="2">
-        <v>0.64583333333333337</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="E37" t="s">
-        <v>51</v>
-      </c>
-      <c r="F37" t="s">
-        <v>13</v>
-      </c>
-      <c r="I37" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C38" s="2">
-        <v>0.64583333333333337</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="D38" s="2">
-        <v>0.66666666666666663</v>
+        <v>0.6875</v>
       </c>
       <c r="E38" t="s">
-        <v>17</v>
+        <v>49</v>
+      </c>
+      <c r="F38" t="s">
+        <v>69</v>
+      </c>
+      <c r="H38" t="s">
+        <v>50</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C39" s="2">
-        <v>0.66666666666666663</v>
+        <v>0.6875</v>
       </c>
       <c r="D39" s="2">
-        <v>0.6875</v>
+        <v>0.70833333333333304</v>
       </c>
       <c r="E39" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F39" t="s">
+        <v>69</v>
+      </c>
+      <c r="H39" t="s">
         <v>63</v>
       </c>
-      <c r="H39" t="s">
-        <v>55</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>73</v>
-      </c>
+      <c r="J39" s="3"/>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>75</v>
+      </c>
       <c r="C40" s="2">
-        <v>0.6875</v>
+        <v>0.375</v>
       </c>
       <c r="D40" s="2">
-        <v>0.70833333333333304</v>
+        <v>0.38541666666666669</v>
       </c>
       <c r="E40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F40" t="s">
+        <v>69</v>
+      </c>
+      <c r="H40" t="s">
         <v>68</v>
       </c>
-      <c r="F40" t="s">
-        <v>63</v>
-      </c>
-      <c r="H40" t="s">
-        <v>74</v>
-      </c>
-      <c r="J40" s="3"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>58</v>
-      </c>
       <c r="C41" s="2">
-        <v>0.375</v>
+        <v>0.38541666666666669</v>
       </c>
       <c r="D41" s="2">
-        <v>0.38541666666666669</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="E41" t="s">
-        <v>52</v>
-      </c>
-      <c r="F41" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="H41" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C42" s="2">
-        <v>0.38541666666666669</v>
+        <v>0.39583333333333298</v>
       </c>
       <c r="D42" s="2">
-        <v>0.39583333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="E42" t="s">
-        <v>78</v>
-      </c>
-      <c r="H42" t="s">
-        <v>77</v>
+        <v>48</v>
+      </c>
+      <c r="F42" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C43" s="2">
-        <v>0.39583333333333298</v>
+        <v>0.5</v>
       </c>
       <c r="D43" s="2">
-        <v>0.5</v>
+        <v>0.54166666666666696</v>
       </c>
       <c r="E43" t="s">
-        <v>53</v>
-      </c>
-      <c r="F43" t="s">
-        <v>63</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="J43" s="3"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C44" s="2">
-        <v>0.5</v>
+        <v>0.54166666666666696</v>
       </c>
       <c r="D44" s="2">
-        <v>0.54166666666666696</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="E44" t="s">
-        <v>20</v>
-      </c>
-      <c r="J44" s="3"/>
+        <v>48</v>
+      </c>
+      <c r="F44" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C45" s="2">
-        <v>0.54166666666666696</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="D45" s="2">
-        <v>0.60416666666666663</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="E45" t="s">
         <v>53</v>
       </c>
       <c r="F45" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C46" s="2">
-        <v>0.60416666666666663</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="D46" s="2">
-        <v>0.66666666666666663</v>
+        <v>0.6875</v>
       </c>
       <c r="E46" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="F46" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C47" s="2">
-        <v>0.66666666666666663</v>
-      </c>
-      <c r="D47" s="2">
-        <v>0.6875</v>
-      </c>
-      <c r="E47" t="s">
-        <v>65</v>
-      </c>
-      <c r="F47" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="H2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="J39" r:id="rId2" xr:uid="{02E4C23A-A3EF-964B-8695-A052AA7101DD}"/>
-    <hyperlink ref="K5" r:id="rId3" xr:uid="{9D7E1F62-7D51-AC46-A470-603E03028633}"/>
+    <hyperlink ref="J38" r:id="rId2" xr:uid="{02E4C23A-A3EF-964B-8695-A052AA7101DD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Schedule: Fix dates and add Tue quiz
</commit_message>
<xml_diff>
--- a/docs/schedule.xlsx
+++ b/docs/schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jenfra/NBISCourses/scRNAseq/workshop-scRNAseq/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8839D084-5412-6946-968E-4FD1A58870D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{989E5B84-3CA6-1B44-9F9B-E5D06AA00DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33700" yWindow="-3400" windowWidth="32200" windowHeight="25700" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19000" yWindow="500" windowWidth="32200" windowHeight="25700" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="80">
   <si>
     <t>date</t>
   </si>
@@ -251,27 +251,12 @@
     <t>27/04/2026</t>
   </si>
   <si>
-    <t>13/04/2025</t>
-  </si>
-  <si>
-    <t>14/04/2025</t>
-  </si>
-  <si>
-    <t>15/04/2025</t>
-  </si>
-  <si>
-    <t>16/04/2025</t>
-  </si>
-  <si>
     <t>Susanne Reinsbach</t>
   </si>
   <si>
     <t>Aditya Singh</t>
   </si>
   <si>
-    <t>Extra time</t>
-  </si>
-  <si>
     <t>Quiz + Extra time</t>
   </si>
   <si>
@@ -282,6 +267,18 @@
   </si>
   <si>
     <t>Guest Lecture: Cell-Cell Communication</t>
+  </si>
+  <si>
+    <t>13/04/2026</t>
+  </si>
+  <si>
+    <t>14/04/2026</t>
+  </si>
+  <si>
+    <t>15/04/2026</t>
+  </si>
+  <si>
+    <t>16/04/2026</t>
   </si>
 </sst>
 </file>
@@ -781,7 +778,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
         <v>51</v>
@@ -932,7 +929,7 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="E11" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F11" t="s">
         <v>64</v>
@@ -941,7 +938,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C12" s="2">
         <v>0.375</v>
@@ -950,7 +947,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J12" s="3"/>
     </row>
@@ -965,7 +962,7 @@
         <v>27</v>
       </c>
       <c r="F13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="H13" t="s">
         <v>28</v>
@@ -994,7 +991,7 @@
         <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="I15" t="s">
         <v>24</v>
@@ -1023,7 +1020,7 @@
         <v>30</v>
       </c>
       <c r="F17" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="H17" t="s">
         <v>31</v>
@@ -1041,7 +1038,7 @@
         <v>32</v>
       </c>
       <c r="F18" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I18" t="s">
         <v>24</v>
@@ -1084,7 +1081,7 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="E21" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F21" t="s">
         <v>64</v>
@@ -1093,7 +1090,7 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="C22" s="2">
         <v>0.375</v>
@@ -1102,7 +1099,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E22" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J22" s="3"/>
     </row>
@@ -1117,7 +1114,7 @@
         <v>35</v>
       </c>
       <c r="F23" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="I23" t="s">
         <v>24</v>
@@ -1176,7 +1173,7 @@
         <v>0.58333333333333304</v>
       </c>
       <c r="E27" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F27" t="s">
         <v>68</v>
@@ -1242,7 +1239,7 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="E31" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F31" t="s">
         <v>64</v>
@@ -1251,7 +1248,7 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C32" s="2">
         <v>0.375</v>
@@ -1260,7 +1257,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E32" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J32" s="3"/>
     </row>
@@ -1364,7 +1361,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="E39" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
replaced integration slides, updated render script and schedule
</commit_message>
<xml_diff>
--- a/docs/schedule.xlsx
+++ b/docs/schedule.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jenfra/NBISCourses/scRNAseq/workshop-scRNAseq/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xsinad/Documents/Codes/workshop-scRNAseq/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{989E5B84-3CA6-1B44-9F9B-E5D06AA00DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F8F0959-B055-5F4F-B16B-B8CA2CA2DD1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19000" yWindow="500" windowWidth="32200" windowHeight="25700" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34560" yWindow="600" windowWidth="32200" windowHeight="25700" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -134,9 +134,6 @@
     <t>Lecture: Batch correction + Integration</t>
   </si>
   <si>
-    <t>lectures/integration.pdf</t>
-  </si>
-  <si>
     <t>Lab: Data integration</t>
   </si>
   <si>
@@ -279,6 +276,9 @@
   </si>
   <si>
     <t>16/04/2026</t>
+  </si>
+  <si>
+    <t>lectures/integration/index.html</t>
   </si>
 </sst>
 </file>
@@ -778,10 +778,10 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C2" s="2">
         <v>0.375</v>
@@ -793,7 +793,7 @@
         <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>14</v>
@@ -808,7 +808,7 @@
         <v>0.4375</v>
       </c>
       <c r="E3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
         <v>18</v>
@@ -869,7 +869,7 @@
         <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H7" t="s">
         <v>22</v>
@@ -887,7 +887,7 @@
         <v>23</v>
       </c>
       <c r="F8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I8" t="s">
         <v>24</v>
@@ -915,7 +915,7 @@
         <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H10" t="s">
         <v>26</v>
@@ -929,16 +929,16 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J11" s="3"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C12" s="2">
         <v>0.375</v>
@@ -947,7 +947,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J12" s="3"/>
     </row>
@@ -962,7 +962,7 @@
         <v>27</v>
       </c>
       <c r="F13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H13" t="s">
         <v>28</v>
@@ -991,7 +991,7 @@
         <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I15" t="s">
         <v>24</v>
@@ -1020,10 +1020,10 @@
         <v>30</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H17" t="s">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="K17" s="3"/>
     </row>
@@ -1035,10 +1035,10 @@
         <v>0.625</v>
       </c>
       <c r="E18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I18" t="s">
         <v>24</v>
@@ -1064,13 +1064,13 @@
         <v>0.6875</v>
       </c>
       <c r="E20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F20" t="s">
         <v>13</v>
       </c>
       <c r="H20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
@@ -1081,16 +1081,16 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="E21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J21" s="3"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C22" s="2">
         <v>0.375</v>
@@ -1099,7 +1099,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J22" s="3"/>
     </row>
@@ -1111,10 +1111,10 @@
         <v>0.4375</v>
       </c>
       <c r="E23" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F23" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I23" t="s">
         <v>24</v>
@@ -1140,16 +1140,16 @@
         <v>0.5</v>
       </c>
       <c r="E25" t="s">
+        <v>35</v>
+      </c>
+      <c r="F25" t="s">
+        <v>53</v>
+      </c>
+      <c r="H25" t="s">
         <v>36</v>
       </c>
-      <c r="F25" t="s">
-        <v>54</v>
-      </c>
-      <c r="H25" t="s">
-        <v>37</v>
-      </c>
       <c r="I25" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K25" s="3"/>
     </row>
@@ -1173,13 +1173,13 @@
         <v>0.58333333333333304</v>
       </c>
       <c r="E27" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H27" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
@@ -1190,16 +1190,16 @@
         <v>0.60416666666666696</v>
       </c>
       <c r="E28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K28" s="3"/>
     </row>
@@ -1222,10 +1222,10 @@
         <v>0.6875</v>
       </c>
       <c r="E30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I30" t="s">
         <v>24</v>
@@ -1239,16 +1239,16 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="E31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F31" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J31" s="3"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C32" s="2">
         <v>0.375</v>
@@ -1257,7 +1257,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E32" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J32" s="3"/>
     </row>
@@ -1269,13 +1269,13 @@
         <v>0.4375</v>
       </c>
       <c r="E33" t="s">
+        <v>39</v>
+      </c>
+      <c r="F33" t="s">
+        <v>54</v>
+      </c>
+      <c r="H33" t="s">
         <v>40</v>
-      </c>
-      <c r="F33" t="s">
-        <v>55</v>
-      </c>
-      <c r="H33" t="s">
-        <v>41</v>
       </c>
       <c r="K33" s="3"/>
     </row>
@@ -1298,10 +1298,10 @@
         <v>0.5</v>
       </c>
       <c r="E35" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F35" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I35" t="s">
         <v>24</v>
@@ -1327,13 +1327,13 @@
         <v>0.58333333333333304</v>
       </c>
       <c r="E37" t="s">
+        <v>42</v>
+      </c>
+      <c r="F37" t="s">
+        <v>65</v>
+      </c>
+      <c r="H37" t="s">
         <v>43</v>
-      </c>
-      <c r="F37" t="s">
-        <v>66</v>
-      </c>
-      <c r="H37" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
@@ -1344,10 +1344,10 @@
         <v>0.63541666666666663</v>
       </c>
       <c r="E38" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I38" t="s">
         <v>24</v>
@@ -1361,7 +1361,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="E39" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
@@ -1383,13 +1383,13 @@
         <v>0.6875</v>
       </c>
       <c r="E41" t="s">
+        <v>47</v>
+      </c>
+      <c r="F41" t="s">
+        <v>63</v>
+      </c>
+      <c r="H41" t="s">
         <v>48</v>
-      </c>
-      <c r="F41" t="s">
-        <v>64</v>
-      </c>
-      <c r="H41" t="s">
-        <v>49</v>
       </c>
       <c r="J41" s="3"/>
     </row>
@@ -1401,19 +1401,19 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="E42" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F42" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J42" s="3"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C43" s="2">
         <v>0.375</v>
@@ -1422,13 +1422,13 @@
         <v>0.38541666666666669</v>
       </c>
       <c r="E43" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F43" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H43" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
@@ -1439,10 +1439,10 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E44" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H44" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
@@ -1453,10 +1453,10 @@
         <v>0.5</v>
       </c>
       <c r="E45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F45" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
@@ -1479,10 +1479,10 @@
         <v>0.60416666666666663</v>
       </c>
       <c r="E47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F47" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
@@ -1493,10 +1493,10 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="E48" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F48" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="49" spans="3:6" x14ac:dyDescent="0.2">
@@ -1507,10 +1507,10 @@
         <v>0.6875</v>
       </c>
       <c r="E49" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Integration Lecture slides (#60)
* replaced integration slides, updated render script and schedule

Incorporates comments: https://github.com/NBISweden/workshop-scRNAseq/pull/60#issuecomment-4075387097

* Better clarification of q18, moved down slide 1:
</commit_message>
<xml_diff>
--- a/docs/schedule.xlsx
+++ b/docs/schedule.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jenfra/NBISCourses/scRNAseq/workshop-scRNAseq/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xsinad/Documents/Codes/workshop-scRNAseq/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{989E5B84-3CA6-1B44-9F9B-E5D06AA00DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F8F0959-B055-5F4F-B16B-B8CA2CA2DD1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19000" yWindow="500" windowWidth="32200" windowHeight="25700" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34560" yWindow="600" windowWidth="32200" windowHeight="25700" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -134,9 +134,6 @@
     <t>Lecture: Batch correction + Integration</t>
   </si>
   <si>
-    <t>lectures/integration.pdf</t>
-  </si>
-  <si>
     <t>Lab: Data integration</t>
   </si>
   <si>
@@ -279,6 +276,9 @@
   </si>
   <si>
     <t>16/04/2026</t>
+  </si>
+  <si>
+    <t>lectures/integration/index.html</t>
   </si>
 </sst>
 </file>
@@ -778,10 +778,10 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C2" s="2">
         <v>0.375</v>
@@ -793,7 +793,7 @@
         <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>14</v>
@@ -808,7 +808,7 @@
         <v>0.4375</v>
       </c>
       <c r="E3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
         <v>18</v>
@@ -869,7 +869,7 @@
         <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H7" t="s">
         <v>22</v>
@@ -887,7 +887,7 @@
         <v>23</v>
       </c>
       <c r="F8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I8" t="s">
         <v>24</v>
@@ -915,7 +915,7 @@
         <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H10" t="s">
         <v>26</v>
@@ -929,16 +929,16 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J11" s="3"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C12" s="2">
         <v>0.375</v>
@@ -947,7 +947,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J12" s="3"/>
     </row>
@@ -962,7 +962,7 @@
         <v>27</v>
       </c>
       <c r="F13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H13" t="s">
         <v>28</v>
@@ -991,7 +991,7 @@
         <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I15" t="s">
         <v>24</v>
@@ -1020,10 +1020,10 @@
         <v>30</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H17" t="s">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="K17" s="3"/>
     </row>
@@ -1035,10 +1035,10 @@
         <v>0.625</v>
       </c>
       <c r="E18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I18" t="s">
         <v>24</v>
@@ -1064,13 +1064,13 @@
         <v>0.6875</v>
       </c>
       <c r="E20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F20" t="s">
         <v>13</v>
       </c>
       <c r="H20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
@@ -1081,16 +1081,16 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="E21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J21" s="3"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C22" s="2">
         <v>0.375</v>
@@ -1099,7 +1099,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J22" s="3"/>
     </row>
@@ -1111,10 +1111,10 @@
         <v>0.4375</v>
       </c>
       <c r="E23" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F23" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I23" t="s">
         <v>24</v>
@@ -1140,16 +1140,16 @@
         <v>0.5</v>
       </c>
       <c r="E25" t="s">
+        <v>35</v>
+      </c>
+      <c r="F25" t="s">
+        <v>53</v>
+      </c>
+      <c r="H25" t="s">
         <v>36</v>
       </c>
-      <c r="F25" t="s">
-        <v>54</v>
-      </c>
-      <c r="H25" t="s">
-        <v>37</v>
-      </c>
       <c r="I25" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K25" s="3"/>
     </row>
@@ -1173,13 +1173,13 @@
         <v>0.58333333333333304</v>
       </c>
       <c r="E27" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H27" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
@@ -1190,16 +1190,16 @@
         <v>0.60416666666666696</v>
       </c>
       <c r="E28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K28" s="3"/>
     </row>
@@ -1222,10 +1222,10 @@
         <v>0.6875</v>
       </c>
       <c r="E30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I30" t="s">
         <v>24</v>
@@ -1239,16 +1239,16 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="E31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F31" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J31" s="3"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C32" s="2">
         <v>0.375</v>
@@ -1257,7 +1257,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E32" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J32" s="3"/>
     </row>
@@ -1269,13 +1269,13 @@
         <v>0.4375</v>
       </c>
       <c r="E33" t="s">
+        <v>39</v>
+      </c>
+      <c r="F33" t="s">
+        <v>54</v>
+      </c>
+      <c r="H33" t="s">
         <v>40</v>
-      </c>
-      <c r="F33" t="s">
-        <v>55</v>
-      </c>
-      <c r="H33" t="s">
-        <v>41</v>
       </c>
       <c r="K33" s="3"/>
     </row>
@@ -1298,10 +1298,10 @@
         <v>0.5</v>
       </c>
       <c r="E35" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F35" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I35" t="s">
         <v>24</v>
@@ -1327,13 +1327,13 @@
         <v>0.58333333333333304</v>
       </c>
       <c r="E37" t="s">
+        <v>42</v>
+      </c>
+      <c r="F37" t="s">
+        <v>65</v>
+      </c>
+      <c r="H37" t="s">
         <v>43</v>
-      </c>
-      <c r="F37" t="s">
-        <v>66</v>
-      </c>
-      <c r="H37" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
@@ -1344,10 +1344,10 @@
         <v>0.63541666666666663</v>
       </c>
       <c r="E38" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I38" t="s">
         <v>24</v>
@@ -1361,7 +1361,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="E39" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
@@ -1383,13 +1383,13 @@
         <v>0.6875</v>
       </c>
       <c r="E41" t="s">
+        <v>47</v>
+      </c>
+      <c r="F41" t="s">
+        <v>63</v>
+      </c>
+      <c r="H41" t="s">
         <v>48</v>
-      </c>
-      <c r="F41" t="s">
-        <v>64</v>
-      </c>
-      <c r="H41" t="s">
-        <v>49</v>
       </c>
       <c r="J41" s="3"/>
     </row>
@@ -1401,19 +1401,19 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="E42" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F42" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J42" s="3"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C43" s="2">
         <v>0.375</v>
@@ -1422,13 +1422,13 @@
         <v>0.38541666666666669</v>
       </c>
       <c r="E43" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F43" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H43" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
@@ -1439,10 +1439,10 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E44" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H44" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
@@ -1453,10 +1453,10 @@
         <v>0.5</v>
       </c>
       <c r="E45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F45" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
@@ -1479,10 +1479,10 @@
         <v>0.60416666666666663</v>
       </c>
       <c r="E47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F47" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
@@ -1493,10 +1493,10 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="E48" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F48" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="49" spans="3:6" x14ac:dyDescent="0.2">
@@ -1507,10 +1507,10 @@
         <v>0.6875</v>
       </c>
       <c r="E49" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: update schedule file dm lecture
</commit_message>
<xml_diff>
--- a/docs/schedule.xlsx
+++ b/docs/schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xsinad/Documents/Codes/workshop-scRNAseq/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/susrei/projects/nbis/workshop-scRNAseq/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F8F0959-B055-5F4F-B16B-B8CA2CA2DD1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E3257D-12FC-C84F-A47F-FE41FF13CFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34560" yWindow="600" windowWidth="32200" windowHeight="25700" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="81">
   <si>
     <t>date</t>
   </si>
@@ -279,6 +279,9 @@
   </si>
   <si>
     <t>lectures/integration/index.html</t>
+  </si>
+  <si>
+    <t>Stephan Nylinder</t>
   </si>
 </sst>
 </file>
@@ -1441,6 +1444,9 @@
       <c r="E44" t="s">
         <v>61</v>
       </c>
+      <c r="F44" t="s">
+        <v>80</v>
+      </c>
       <c r="H44" t="s">
         <v>60</v>
       </c>

</xml_diff>

<commit_message>
fixups: making pre launch changes (#61)
* scanpy: update instructions

* docs: update schedule file dm lecture

* spatial: remove labs and references

* containers/seurat: accept conda tos

* compiled/seurat: minor formatting fix qc

* docs/labs/scanpy: update trajectory

* docs/labs/scanpy: set random state

* docs/labs/scanpy: fix download celltyping

* docs/labs/scanpy: gsea error handling

* docs/labs/scanpy: bug fixes trajectory

* docs/labs/scanpy: formatting trajectory

* compiled/scanpy: update labs

* docs: fixes to colima instructions

* docs/quarto: add 2025 archive entry

---------

Co-authored-by: Stefan Ebmeyer <stefan.ebmeyer@scilifelab.se>
</commit_message>
<xml_diff>
--- a/docs/schedule.xlsx
+++ b/docs/schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xsinad/Documents/Codes/workshop-scRNAseq/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/susrei/projects/nbis/workshop-scRNAseq/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F8F0959-B055-5F4F-B16B-B8CA2CA2DD1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E3257D-12FC-C84F-A47F-FE41FF13CFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34560" yWindow="600" windowWidth="32200" windowHeight="25700" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="81">
   <si>
     <t>date</t>
   </si>
@@ -279,6 +279,9 @@
   </si>
   <si>
     <t>lectures/integration/index.html</t>
+  </si>
+  <si>
+    <t>Stephan Nylinder</t>
   </si>
 </sst>
 </file>
@@ -1441,6 +1444,9 @@
       <c r="E44" t="s">
         <v>61</v>
       </c>
+      <c r="F44" t="s">
+        <v>80</v>
+      </c>
       <c r="H44" t="s">
         <v>60</v>
       </c>

</xml_diff>

<commit_message>
Remove dge and gsa pdfs, add CCC pdf
</commit_message>
<xml_diff>
--- a/docs/schedule.xlsx
+++ b/docs/schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/susrei/projects/nbis/workshop-scRNAseq/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jenfra/NBISCourses/scRNAseq/workshop-scRNAseq/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E3257D-12FC-C84F-A47F-FE41FF13CFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A9117BF-ADE5-034F-986B-B293A87A2CED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="79">
   <si>
     <t>date</t>
   </si>
@@ -213,12 +213,6 @@
   </si>
   <si>
     <t>lectures/preBYOD.pdf</t>
-  </si>
-  <si>
-    <t>lectures/dge.pdf</t>
-  </si>
-  <si>
-    <t>lectures/gsa.pdf</t>
   </si>
   <si>
     <t>lectures/DataManagement.pdf</t>
@@ -781,7 +775,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s">
         <v>50</v>
@@ -796,7 +790,7 @@
         <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>14</v>
@@ -872,7 +866,7 @@
         <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H7" t="s">
         <v>22</v>
@@ -918,7 +912,7 @@
         <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H10" t="s">
         <v>26</v>
@@ -932,16 +926,16 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J11" s="3"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C12" s="2">
         <v>0.375</v>
@@ -950,7 +944,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J12" s="3"/>
     </row>
@@ -965,7 +959,7 @@
         <v>27</v>
       </c>
       <c r="F13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H13" t="s">
         <v>28</v>
@@ -994,7 +988,7 @@
         <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I15" t="s">
         <v>24</v>
@@ -1023,10 +1017,10 @@
         <v>30</v>
       </c>
       <c r="F17" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H17" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="K17" s="3"/>
     </row>
@@ -1041,7 +1035,7 @@
         <v>31</v>
       </c>
       <c r="F18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I18" t="s">
         <v>24</v>
@@ -1084,16 +1078,16 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="E21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F21" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J21" s="3"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C22" s="2">
         <v>0.375</v>
@@ -1102,7 +1096,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E22" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J22" s="3"/>
     </row>
@@ -1117,7 +1111,7 @@
         <v>34</v>
       </c>
       <c r="F23" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I23" t="s">
         <v>24</v>
@@ -1151,9 +1145,6 @@
       <c r="H25" t="s">
         <v>36</v>
       </c>
-      <c r="I25" t="s">
-        <v>58</v>
-      </c>
       <c r="K25" s="3"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
@@ -1176,13 +1167,13 @@
         <v>0.58333333333333304</v>
       </c>
       <c r="E27" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F27" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H27" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
@@ -1201,9 +1192,6 @@
       <c r="H28" t="s">
         <v>49</v>
       </c>
-      <c r="I28" t="s">
-        <v>59</v>
-      </c>
       <c r="K28" s="3"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
@@ -1242,16 +1230,16 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="E31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F31" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J31" s="3"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C32" s="2">
         <v>0.375</v>
@@ -1260,7 +1248,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E32" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J32" s="3"/>
     </row>
@@ -1333,7 +1321,7 @@
         <v>42</v>
       </c>
       <c r="F37" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H37" t="s">
         <v>43</v>
@@ -1350,7 +1338,7 @@
         <v>44</v>
       </c>
       <c r="F38" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I38" t="s">
         <v>24</v>
@@ -1364,7 +1352,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="E39" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
@@ -1389,7 +1377,7 @@
         <v>47</v>
       </c>
       <c r="F41" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H41" t="s">
         <v>48</v>
@@ -1407,7 +1395,7 @@
         <v>55</v>
       </c>
       <c r="F42" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H42" t="s">
         <v>57</v>
@@ -1416,7 +1404,7 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C43" s="2">
         <v>0.375</v>
@@ -1428,10 +1416,10 @@
         <v>45</v>
       </c>
       <c r="F43" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H43" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
@@ -1442,13 +1430,13 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E44" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F44" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H44" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
@@ -1462,7 +1450,7 @@
         <v>46</v>
       </c>
       <c r="F45" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
@@ -1488,7 +1476,7 @@
         <v>46</v>
       </c>
       <c r="F47" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
@@ -1502,7 +1490,7 @@
         <v>51</v>
       </c>
       <c r="F48" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="49" spans="3:6" x14ac:dyDescent="0.2">
@@ -1516,7 +1504,7 @@
         <v>52</v>
       </c>
       <c r="F49" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>